<commit_message>
Refactor AgeGroupService and GroupService to improve data parsing; update AgeGroup and Group models for better property access
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henkelmath\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3559476-2FFF-4D01-AF4E-A0BE9893F216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110F5C56-EC92-4F87-9E41-A32C03A511FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>Lehrjahr</t>
   </si>
@@ -51,6 +51,18 @@
   </si>
   <si>
     <t>FI26a</t>
+  </si>
+  <si>
+    <t>Schulwochen</t>
+  </si>
+  <si>
+    <t>FI26b</t>
+  </si>
+  <si>
+    <t>2. Lj</t>
+  </si>
+  <si>
+    <t>FI25a</t>
   </si>
 </sst>
 </file>
@@ -428,28 +440,201 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA7A25F-1A13-43E6-8B5A-038B5C3A6F73}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" customWidth="1"/>
-    <col min="3" max="3" width="29.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" customWidth="1"/>
+    <col min="3" max="3" width="29.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="C3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="C4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="C5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="C6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="C7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="C8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="C9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="B10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="C12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="C13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="C14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="C15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="C16">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="C17">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="C19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="C20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="C21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="C22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="C23">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="C24">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="C25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="B26" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="C27">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="C28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="C29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="C30">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="C31">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="C32">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added blocks to Groups. Started Adding parsing blocks from excel tables.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8ADC219-5D68-4643-AA15-D25D569027A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F125B611-9FF8-4035-86FB-B39D70C18B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
@@ -136,9 +136,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -511,13 +514,13 @@
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>10</v>
       </c>
       <c r="F2" t="s">
@@ -525,13 +528,13 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="C3">
+      <c r="C3" s="2">
         <v>2</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>4</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -539,13 +542,13 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="C4">
+      <c r="C4" s="2">
         <v>3</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>4</v>
       </c>
       <c r="F4" t="s">
@@ -553,44 +556,49 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="C5">
+      <c r="C5" s="2">
         <v>4</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
       </c>
+      <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="C6">
+      <c r="C6" s="2">
         <v>5</v>
       </c>
+      <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="C7">
+      <c r="C7" s="2">
         <v>6</v>
       </c>
+      <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="C8">
+      <c r="C8" s="2">
         <v>8</v>
       </c>
+      <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="C9">
+      <c r="C9" s="2">
         <v>9</v>
       </c>
+      <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="2">
         <v>1</v>
       </c>
       <c r="D10" t="s">
         <v>14</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>10</v>
       </c>
       <c r="F10" t="s">
@@ -598,13 +606,13 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="C11">
+      <c r="C11" s="2">
         <v>2</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="2">
         <v>4</v>
       </c>
       <c r="F11" s="1" t="s">
@@ -612,13 +620,13 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="C12">
+      <c r="C12" s="2">
         <v>3</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>4</v>
       </c>
       <c r="F12" t="s">
@@ -626,35 +634,39 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="C13">
+      <c r="C13" s="2">
         <v>4</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="C14">
+      <c r="C14" s="2">
         <v>5</v>
       </c>
+      <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="C15">
+      <c r="C15" s="2">
         <v>6</v>
       </c>
+      <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="C16">
+      <c r="C16" s="2">
         <v>8</v>
       </c>
+      <c r="E16" s="2"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="C17">
+      <c r="C17" s="2">
         <v>9</v>
       </c>
+      <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
@@ -663,13 +675,13 @@
       <c r="B18" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="2">
         <v>1</v>
       </c>
       <c r="D18" t="s">
         <v>15</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="2">
         <v>2</v>
       </c>
       <c r="F18" t="s">
@@ -677,13 +689,13 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="C19">
+      <c r="C19" s="2">
         <v>2</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="2">
         <v>2</v>
       </c>
       <c r="F19" s="1" t="s">
@@ -691,13 +703,13 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="C20">
+      <c r="C20" s="2">
         <v>3</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="2">
         <v>4</v>
       </c>
       <c r="F20" t="s">
@@ -705,7 +717,7 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="C21">
+      <c r="C21" s="2">
         <v>4</v>
       </c>
       <c r="D21" t="s">
@@ -713,7 +725,7 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="C22">
+      <c r="C22" s="2">
         <v>5</v>
       </c>
       <c r="D22" t="s">
@@ -721,17 +733,17 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="C23">
+      <c r="C23" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="C24">
+      <c r="C24" s="2">
         <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="C25">
+      <c r="C25" s="2">
         <v>9</v>
       </c>
     </row>
@@ -739,42 +751,42 @@
       <c r="B26" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="C27">
+      <c r="C27" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="C28">
+      <c r="C28" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="C29">
+      <c r="C29" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="C30">
+      <c r="C30" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="C31">
+      <c r="C31" s="2">
         <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:6">
-      <c r="C32">
+      <c r="C32" s="2">
         <v>8</v>
       </c>
     </row>
     <row r="33" spans="3:3">
-      <c r="C33">
+      <c r="C33" s="2">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Split each IEntityService into an IConfigService and and IEntityService. IConfigServices now read basic configuration infromation from ecxel files. IEntityServices should build complex objets from the configuration data.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F125B611-9FF8-4035-86FB-B39D70C18B7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9840675-1A8C-4C27-BB7D-7FB722771C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="11940" yWindow="0" windowWidth="15180" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
   <si>
     <t>Lehrjahr</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>Pruefungsvorbereitung</t>
+  </si>
+  <si>
+    <t>FI25b</t>
   </si>
 </sst>
 </file>
@@ -562,7 +565,9 @@
       <c r="D5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2">
+        <v>6</v>
+      </c>
     </row>
     <row r="6" spans="1:6">
       <c r="C6" s="2">
@@ -723,6 +728,9 @@
       <c r="D21" t="s">
         <v>17</v>
       </c>
+      <c r="E21" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="22" spans="1:6">
       <c r="C22" s="2">
@@ -731,6 +739,9 @@
       <c r="D22" t="s">
         <v>18</v>
       </c>
+      <c r="E22" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="23" spans="1:6">
       <c r="C23" s="2">
@@ -749,7 +760,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="B26" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="C26" s="2">
         <v>1</v>

</xml_diff>

<commit_message>
Made cards in edit view actually data driven.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9840675-1A8C-4C27-BB7D-7FB722771C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{362C507D-CFDD-435B-A0BB-84E9B824A068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11940" yWindow="0" windowWidth="15180" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="13650" yWindow="720" windowWidth="15180" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="20">
   <si>
     <t>Lehrjahr</t>
   </si>
@@ -573,19 +573,34 @@
       <c r="C6" s="2">
         <v>5</v>
       </c>
-      <c r="E6" s="2"/>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2">
+        <v>6</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
       <c r="C7" s="2">
         <v>6</v>
       </c>
-      <c r="E7" s="2"/>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="2">
+        <v>6</v>
+      </c>
     </row>
     <row r="8" spans="1:6">
       <c r="C8" s="2">
         <v>8</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="2">
+        <v>6</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="C9" s="2">

</xml_diff>

<commit_message>
Added a teacher to each group. Updated GeneratorService. Cleanded up GroupService. Updated Lehrjahre.xlsx.
</commit_message>
<xml_diff>
--- a/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
+++ b/EinsatzPlanung/Assets/Excel/Lehrjahre.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\EinsatzPlanung\EinsatzPlanung\Assets\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{362C507D-CFDD-435B-A0BB-84E9B824A068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41E6D75-EC3B-491D-872A-E8A21199EA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13650" yWindow="720" windowWidth="15180" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
+    <workbookView xWindow="150" yWindow="690" windowWidth="23925" windowHeight="15645" xr2:uid="{93971DC9-9131-4D11-831F-804A5976373C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
   <si>
     <t>Lehrjahr</t>
   </si>
@@ -99,6 +99,18 @@
   </si>
   <si>
     <t>FI25b</t>
+  </si>
+  <si>
+    <t>Ausbilder</t>
+  </si>
+  <si>
+    <t>He</t>
+  </si>
+  <si>
+    <t>Lu</t>
+  </si>
+  <si>
+    <t>Sch</t>
   </si>
 </sst>
 </file>
@@ -479,18 +491,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA7A25F-1A13-43E6-8B5A-038B5C3A6F73}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -498,321 +510,336 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
-      <c r="C3" s="2">
+    <row r="3" spans="1:7">
+      <c r="D3" s="2">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="2">
-        <v>4</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2">
+        <v>4</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
-      <c r="C4" s="2">
+    <row r="4" spans="1:7">
+      <c r="D4" s="2">
         <v>3</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="2">
-        <v>4</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2">
+        <v>4</v>
+      </c>
+      <c r="G4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="C5" s="2">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
+    <row r="5" spans="1:7">
+      <c r="D5" s="2">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
-      <c r="C6" s="2">
+    <row r="6" spans="1:7">
+      <c r="D6" s="2">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
-      <c r="C7" s="2">
+    <row r="7" spans="1:7">
+      <c r="D7" s="2">
         <v>6</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
-      <c r="C8" s="2">
+    <row r="8" spans="1:7">
+      <c r="D8" s="2">
         <v>8</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
-      <c r="C9" s="2">
+    <row r="9" spans="1:7">
+      <c r="D9" s="2">
         <v>9</v>
       </c>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:7">
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2">
         <v>1</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="2">
         <v>10</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
-      <c r="C11" s="2">
+    <row r="11" spans="1:7">
+      <c r="D11" s="2">
         <v>2</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="2">
-        <v>4</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="2">
+        <v>4</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="C12" s="2">
+    <row r="12" spans="1:7">
+      <c r="D12" s="2">
         <v>3</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="2">
-        <v>4</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2">
+        <v>4</v>
+      </c>
+      <c r="G12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
-      <c r="C13" s="2">
-        <v>4</v>
-      </c>
-      <c r="D13" t="s">
+    <row r="13" spans="1:7">
+      <c r="D13" s="2">
+        <v>4</v>
+      </c>
+      <c r="E13" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="C14" s="2">
+    <row r="14" spans="1:7">
+      <c r="D14" s="2">
         <v>5</v>
       </c>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="C15" s="2">
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="D15" s="2">
         <v>6</v>
       </c>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="C16" s="2">
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="D16" s="2">
         <v>8</v>
       </c>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="C17" s="2">
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="D17" s="2">
         <v>9</v>
       </c>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>6</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="2">
         <v>1</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="2">
+      <c r="F18" s="2">
         <v>2</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
-      <c r="C19" s="2">
+    <row r="19" spans="1:7">
+      <c r="D19" s="2">
         <v>2</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>11</v>
       </c>
-      <c r="E19" s="2">
+      <c r="F19" s="2">
         <v>2</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
-      <c r="C20" s="2">
+    <row r="20" spans="1:7">
+      <c r="D20" s="2">
         <v>3</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="E20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="2">
-        <v>4</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="F20" s="2">
+        <v>4</v>
+      </c>
+      <c r="G20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
-      <c r="C21" s="2">
-        <v>4</v>
-      </c>
-      <c r="D21" t="s">
+    <row r="21" spans="1:7">
+      <c r="D21" s="2">
+        <v>4</v>
+      </c>
+      <c r="E21" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="C22" s="2">
+      <c r="F21" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="D22" s="2">
         <v>5</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>18</v>
       </c>
-      <c r="E22" s="2">
+      <c r="F22" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
-      <c r="C23" s="2">
+    <row r="23" spans="1:7">
+      <c r="D23" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
-      <c r="C24" s="2">
+    <row r="24" spans="1:7">
+      <c r="D24" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
-      <c r="C25" s="2">
+    <row r="25" spans="1:7">
+      <c r="D25" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:7">
       <c r="B26" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
-      <c r="C27" s="2">
+    <row r="27" spans="1:7">
+      <c r="D27" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
-      <c r="C28" s="2">
+    <row r="28" spans="1:7">
+      <c r="D28" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
-      <c r="C29" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="C30" s="2">
+    <row r="29" spans="1:7">
+      <c r="D29" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="D30" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
-      <c r="C31" s="2">
+    <row r="31" spans="1:7">
+      <c r="D31" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
-      <c r="C32" s="2">
+    <row r="32" spans="1:7">
+      <c r="D32" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="3:3">
-      <c r="C33" s="2">
+    <row r="33" spans="4:4">
+      <c r="D33" s="2">
         <v>9</v>
       </c>
     </row>

</xml_diff>